<commit_message>
testdata update for git actions
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C788A72E-5A68-45A6-ADFF-12E1E360CE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC5F383-4DDB-4B9D-B1C9-08FC82CBB24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,10 +108,10 @@
     <t>Andhra</t>
   </si>
   <si>
-    <t>prasad153</t>
-  </si>
-  <si>
-    <t>testuser153@yopmail.com</t>
+    <t>prasad246</t>
+  </si>
+  <si>
+    <t>testuser246@yopmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
update workflow with Azure
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F5D4E7-47DA-4811-A9D4-401C84CAB400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B713BEE-6275-4D82-83B3-B93ABA4FCDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Name</t>
   </si>
@@ -108,16 +108,10 @@
     <t>Andhra</t>
   </si>
   <si>
-    <t>gvvtest71992</t>
-  </si>
-  <si>
-    <t>gvvtest5670@yopmail.com</t>
-  </si>
-  <si>
-    <t>gvvtest10992@yopmail.com</t>
-  </si>
-  <si>
-    <t>gvvtest74040</t>
+    <t>gvvtest71933</t>
+  </si>
+  <si>
+    <t>gvvtest9671@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -446,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
@@ -572,65 +566,10 @@
         <v>9977551133</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3">
-        <v>23</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3">
-        <v>2000</v>
-      </c>
-      <c r="J3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" t="s">
-        <v>26</v>
-      </c>
-      <c r="O3" t="s">
-        <v>25</v>
-      </c>
-      <c r="P3">
-        <v>500335</v>
-      </c>
-      <c r="Q3">
-        <v>9977551133</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{D6A3B950-DB4D-483C-A98B-15EE16C9FA39}"/>
     <hyperlink ref="F2" r:id="rId2" xr:uid="{851D07DC-EC92-4332-AB7B-07EC8056F930}"/>
-    <hyperlink ref="D3" r:id="rId3" xr:uid="{4D2B3D44-0F7E-46B5-ACE0-D722AEA02DBB}"/>
-    <hyperlink ref="F3" r:id="rId4" xr:uid="{029352C1-01BF-48E4-9A4A-2400EDF19CB2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
validaing product details page
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A296FA1-E5B7-45C1-A6BF-4A1E5DBA03C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4FB02D-3296-4D41-A087-046F63D1968B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -115,9 +115,6 @@
     <t>kakinada</t>
   </si>
   <si>
-    <t>gvv5</t>
-  </si>
-  <si>
     <t>gvv9</t>
   </si>
   <si>
@@ -125,9 +122,6 @@
   </si>
   <si>
     <t>Negative</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Yes</t>
@@ -483,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.44140625" customWidth="1"/>
@@ -559,16 +553,16 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="E2" t="s">
         <v>23</v>
@@ -612,22 +606,19 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G3">
         <v>23</v>
@@ -638,69 +629,18 @@
       <c r="I3">
         <v>1990</v>
       </c>
-      <c r="J3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" t="s">
-        <v>26</v>
-      </c>
       <c r="L3" t="s">
         <v>21</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" t="s">
-        <v>27</v>
-      </c>
-      <c r="O3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P3">
-        <v>500335</v>
-      </c>
-      <c r="Q3">
-        <v>9988774455</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4">
-        <v>1990</v>
-      </c>
-      <c r="L4" t="s">
-        <v>21</v>
-      </c>
-      <c r="M4" t="s">
         <v>22</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{09D6043E-1C09-4C93-9C5F-D090433018DF}"/>
-    <hyperlink ref="D3" r:id="rId2" display="gvv5@yopmail.com" xr:uid="{69C525D9-A1AC-4A99-8E3C-E1F95DCB80C8}"/>
-    <hyperlink ref="D2" r:id="rId3" xr:uid="{87E608F6-2070-4106-B3C4-E355E5CB1189}"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{09D6043E-1C09-4C93-9C5F-D090433018DF}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{87E608F6-2070-4106-B3C4-E355E5CB1189}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -735,36 +675,36 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>35</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Tests related to cart and updated the naming conventions
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4FB02D-3296-4D41-A087-046F63D1968B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECD7177-B1DE-48A1-99CA-E6932BDA84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
     <sheet name="login" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
   <si>
     <t>Name</t>
   </si>
@@ -143,6 +144,9 @@
   </si>
   <si>
     <t>gvvtest1</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
@@ -714,4 +718,28 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE99E6B8-824C-4732-B2C5-23DC1F2D6217}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
comments added & extra spaces removed
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECD7177-B1DE-48A1-99CA-E6932BDA84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8778F3-EE48-4FF9-9D60-BD8E6B5DD7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
     <sheet name="login" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="products" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="44">
   <si>
     <t>Name</t>
   </si>
@@ -147,6 +147,18 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>Men Tshirt</t>
+  </si>
+  <si>
+    <t>Sleeveless Dress</t>
+  </si>
+  <si>
+    <t>Stylish Dress</t>
+  </si>
+  <si>
+    <t>Premium Polo T-Shirts</t>
   </si>
 </sst>
 </file>
@@ -722,8 +734,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE99E6B8-824C-4732-B2C5-23DC1F2D6217}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -739,6 +754,62 @@
         <v>39</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
code optimized of gvv branch
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECD7177-B1DE-48A1-99CA-E6932BDA84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD160EE6-1C6C-419C-ACA0-0B1817D81A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
@@ -481,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.44140625" customWidth="1"/>
@@ -639,6 +639,9 @@
       <c r="M3" t="s">
         <v>22</v>
       </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D4" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>